<commit_message>
Refresh seed from the live admin export; fix About text and Projects menu
- fixtures/seed_data.xlsx: replace with the 2026-09-25 admin export, which is
  more current than the old baseline (content was edited by hand in the admin).
- AboutPage: match text sizes used on other pages and justify descriptive text.
- Projects mega menu (desktop + mobile): list every active category instead of
  only beekeeping/environment/ohs, so Agriculture is no longer hidden.
- Category icons: pick one that suits the name; the pin is only the last resort
  (Icon was turning every emoji into the fallback pin).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017ZEn6xMPZAgVcAm9EZYYLS
</commit_message>
<xml_diff>
--- a/fixtures/seed_data.xlsx
+++ b/fixtures/seed_data.xlsx
@@ -720,7 +720,11 @@
           <t>:shield:</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>media/consultation_categories/WhatsApp_Image_2026-09-25_at_08.59.20_xvkoxd</t>
+        </is>
+      </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
@@ -1745,17 +1749,18 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>FEE-VERT Solution Limited is a Tanzanian consultancy specializing in environmental management, sustainable agriculture &amp; commercial beekeeping, and Occupational Health &amp; Safety (OHS). Our multidisciplinary team delivers practical, compliant, and sustainable solutions for public and private sector clients.</t>
+          <t>FEE-VERT Solution Limited is an integrated environmental and agribusiness consultancy firm based in Dar es Salaam, Tanzania, founded in 2015.
+The company offers environmental management services, including Environmental Impact Assessment (EIA), environmental compliance audits, and rehabilitation plans. It also provides Occupational Health and Safety (OHS) services, including safety audits, training, and monitoring, as well as agribusiness support, including agricultural farming management, beekeeping training, and value addition.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Is to provide innovative, reliable, and sustainable professional solutions in Environmental Management, Agriculture, Occupational Health &amp; Safety (OHS), and related technical services that create lasting value for our clients, communities, and the environment.</t>
+          <t>To empower business and communities through expert consultancy that drives sustainable growth and environmental stewardship.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>To become a leading provider of sustainable environmental, agricultural, and occupational health and safety solutions, recognized for excellence, innovation, integrity, and positive impact across Africa.</t>
+          <t>To be Tanzania’s most trusted consultancy partner, recognized for excellence in environmental protection, workplace safety, and agricultural innovation.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
@@ -3541,7 +3546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R16"/>
+  <dimension ref="A1:R15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3671,36 +3676,76 @@
       <c r="H2" t="b">
         <v>1</v>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>ESIA</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Linda idhini zako kwa kujiamini. Huduma yetu ya Tathmini ya Athari kwa Mazingira na Kijamii (ESIA) hutambua athari za mradi kwa mazingira na kijamii mapema - na kuzigeuza kuwa mpango wazi wa usimamizi unaotekelezeka. Tunashughulikia tafiti za kimsingi, mashauriano ya washikadau, ubashiri wa athari na muundo wa kupunguza, na kuandaa hati zilizo tayari za NEMC ambazo hudumisha mradi wako utii, wa kuaminika na kwa ratiba. Iwe unaunda mgodi, kiwanda au mradi wa miundombinu, tunakusaidia kupata kibali na kulinda sifa yako.</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>EIES</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Sécurisez vos approbations en toute confiance. Notre service d'évaluation de l'impact environnemental et social (EIES) identifie très tôt les impacts environnementaux et sociaux d'un projet et les transforme en un plan de gestion clair et réalisable. Nous gérons les études de base, la consultation des parties prenantes, la prévision des impacts et la conception de l'atténuation, et préparons une documentation prête pour le NEMC qui maintient votre projet conforme, crédible et dans les délais. Que vous développiez une mine, une usine ou un projet d'infrastructure, nous vous aidons à obtenir l'approbation et à protéger votre réputation.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>تقييم الأثر البيئي والاجتماعي</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>قم بتأمين الموافقات الخاصة بك بثقة. تحدد خدمة تقييم الأثر البيئي والاجتماعي (ESIA) لدينا الآثار البيئية والاجتماعية للمشروع مبكرًا - وتحولها إلى خطة إدارة واضحة وقابلة للتنفيذ. نحن نتعامل مع الدراسات الأساسية، ومشاورة أصحاب المصلحة، والتنبؤ بالتأثير وتصميم التخفيف، وإعداد وثائق جاهزة لـ NEMC تحافظ على امتثال مشروعك ومصداقيته وفي الموعد المحدد. سواء كنت تقوم بتطوير منجم أو مصنع أو مشروع بنية تحتية، فإننا نساعدك على الحصول على الموافقة وحماية سمعتك.</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>ОВОСС</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Обеспечьте свое одобрение с уверенностью. Наша служба оценки экологического и социального воздействия (ESIA) заранее определяет экологические и социальные последствия проекта и превращает их в четкий и действенный план управления. Мы проводим базовые исследования, консультации с заинтересованными сторонами, прогнозируем воздействие и разрабатываем меры по смягчению последствий, а также подготавливаем документацию, готовую для NEMC, которая обеспечивает соответствие вашего проекта, достоверность и соблюдение графика. Независимо от того, разрабатываете ли вы шахту, завод или инфраструктурный проект, мы поможем вам получить одобрение и защитить вашу репутацию.</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>环境影响评估</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>放心地获得您的批准。我们的环境和社会影响评估 (ESIA) 服务尽早确定项目的环境和社会影响，并将其转化为清晰、可操作的管理计划。我们处理基线研究、利益相关者咨询、影响预测和缓解设计，并准备 NEMC 就绪文档，使您的项目合规、可信并按计划进行。无论您是开发矿山、工厂还是基础设施项目，我们都能帮助您赢得批准并保护您的声誉。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Environmental Auditing</t>
+          <t>Risk Assessment</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>environmental-auditing</t>
+          <t>risk-assessment</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Stay ahead of compliance risks. Our independent environmental audits give you an honest, expert picture of how your operations measure up against environmental laws, permit conditions and your own management plans. We identify gaps before regulators do, quantify your risks, and deliver practical, prioritised corrective actions. The result is a stronger licence to operate, fewer surprises, and a demonstrable commitment to environmental responsibility.</t>
+          <t>Protect your people and your productivity. Our thorough workplace risk assessments uncover hidden hazards and deliver practical controls that prevent incidents before they happen. We systematically identify, evaluate and prioritise risks across your operations, then recommend cost-effective measures that keep workers safe and operations running. Reduce accidents, lower costs, and demonstrate genuine care for your workforce.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>📋</t>
+          <t>⚠️</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -3708,45 +3753,85 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>environment</t>
+          <t>ohs</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H3" t="b">
         <v>1</v>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Tathmini ya Hatari</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Linda watu wako na tija yako. Tathmini zetu za kina za hatari za mahali pa kazi hufichua hatari zilizofichwa na kutoa udhibiti wa vitendo ambao huzuia matukio kabla hayajatokea. Tunatambua, kutathmini na kuzipa kipaumbele hatari katika shughuli zako zote, kisha tunapendekeza hatua za gharama nafuu zinazowaweka wafanyakazi salama na shughuli zinaendelea. Punguza ajali, punguza gharama, na uonyeshe utunzaji wa kweli kwa wafanyikazi wako.</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>L'évaluation des risques</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Protégez vos collaborateurs et votre productivité. Nos évaluations approfondies des risques sur le lieu de travail révèlent les dangers cachés et fournissent des contrôles pratiques qui préviennent les incidents avant qu'ils ne surviennent. Nous identifions, évaluons et hiérarchisons systématiquement les risques dans vos opérations, puis recommandons des mesures rentables qui assurent la sécurité des travailleurs et le bon fonctionnement des opérations. Réduisez les accidents, réduisez les coûts et faites preuve d’une véritable attention envers votre main-d’œuvre.</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>تقييم المخاطر</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>حماية موظفيك وإنتاجيتك. تكشف تقييماتنا الشاملة للمخاطر في مكان العمل عن المخاطر الخفية وتوفر ضوابط عملية تمنع وقوع الحوادث قبل وقوعها. نحن نقوم بتحديد المخاطر وتقييمها وترتيب أولوياتها بشكل منهجي عبر عملياتك، ثم نوصي بإجراءات فعالة من حيث التكلفة تحافظ على سلامة العمال وتشغيل العمليات. يمكنك تقليل الحوادث وخفض التكاليف وإظهار الرعاية الحقيقية للقوى العاملة لديك.</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Оценка риска</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Защитите своих сотрудников и свою производительность. Наши тщательные оценки рисков на рабочем месте выявляют скрытые опасности и обеспечивают практический контроль, предотвращающий инциденты до того, как они произойдут. Мы систематически выявляем, оцениваем и приоритизируем риски в ваших операциях, а затем рекомендуем экономически эффективные меры, обеспечивающие безопасность работников и бесперебойную работу операций. Сократите количество несчастных случаев, снизьте затраты и продемонстрируйте искреннюю заботу о своих сотрудниках.</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>风险评估</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>保护您的员工和您的生产力。我们彻底的工作场所风险评估可以发现隐藏的危险，并提供切实可行的控制措施，防患于未然。我们系统地识别、评估您运营中的风险并确定优先级，然后提出具有成本效益的措施，以确保员工安全和运营正常运行。减少事故、降低成本并表现出对员工的真诚关怀。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mine Closure &amp; Rehabilitation Plan</t>
+          <t>Apiary Establishment &amp; Management</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>mine-closure-rehabilitation</t>
+          <t>apiary-establishment-management</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Close responsibly and protect your legacy. We design practical, regulator-approved mine closure and rehabilitation plans that meet your legal obligations while restoring land the community can trust. Our team addresses landform design, revegetation, water management and post-closure monitoring, with realistic cost estimates you can plan around. Start planning early with us and turn closure from a liability into a well-managed, credible commitment.</t>
+          <t>Start your apiary the right way and keep it thriving. We handle everything from expert site selection and hive installation to colony management, pest and disease control, and ongoing maintenance — so your bees stay healthy and your harvests stay strong, season after season. Whether you are starting fresh or scaling up, we build and run productive apiaries you can rely on.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>⛏️</t>
+          <t>🐝</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -3754,45 +3839,85 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>environment</t>
+          <t>beekeeping</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H4" t="b">
         <v>1</v>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Uanzishaji na Usimamizi wa Hifadhi ya Ndege</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Anzisha nyumba yako ya kuhifadhia wanyama kwa njia sahihi na iendelee kustawi. Tunashughulikia kila kitu kuanzia uteuzi wa tovuti wa wataalam na uwekaji wa mizinga hadi udhibiti wa makundi, udhibiti wa wadudu na magonjwa, na matengenezo yanayoendelea - ili nyuki wako wawe na afya nzuri na mavuno yako yaendelee kuwa na nguvu, msimu baada ya msimu. Iwe unaanza upya au unaongeza kasi, tunaunda na kuendesha apiaries za uzalishaji ambazo unaweza kutegemea.</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Création et gestion d'un rucher</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Démarrez votre rucher de la bonne manière et continuez à prospérer. Nous nous occupons de tout, de la sélection experte du site et de l'installation des ruches à la gestion des colonies, au contrôle des parasites et des maladies et à l'entretien continu — afin que vos abeilles restent en bonne santé et que vos récoltes restent fortes, saison après saison. Que vous démarriez à zéro ou que vous passiez à une plus grande échelle, nous construisons et gérons des ruchers productifs sur lesquels vous pouvez compter.</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>إنشاء وإدارة المنحل</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>ابدأ المنحل الخاص بك بالطريقة الصحيحة وحافظ عليه مزدهرًا. نحن نتعامل مع كل شيء بدءًا من اختيار موقع الخبراء وتركيب الخلية وحتى إدارة المستعمرة ومكافحة الآفات والأمراض والصيانة المستمرة - حتى يظل النحل في صحة جيدة ويظل حصادك قويًا، موسمًا بعد موسم. سواء كنت تبدأ نشاطًا جديدًا أو تقوم بتوسيع نطاق أعمالك، فإننا نبني وندير مناحل منتجة يمكنك الاعتماد عليها.</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Создание и управление пасекой</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Начните свою пасеку правильно и поддерживайте ее процветание. Мы занимаемся всем: от профессионального выбора места и установки ульев до управления семьями, борьбы с вредителями и болезнями, а также текущего обслуживания — чтобы ваши пчелы оставались здоровыми, а ваши урожаи — сильными, сезон за сезоном. Независимо от того, начинаете ли вы с нуля или расширяете масштабы деятельности, мы создаем и управляем продуктивными пасеками, на которые вы можете положиться.</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>养蜂场的建立和管理</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>以正确的方式开始您的养蜂场并使其蓬勃发展。我们负责处理从专家选址和蜂巢安装到蜂群管理、病虫害控制以及持续维护的一切事宜，让您的蜜蜂保持健康，让您的收成保持旺盛。无论您是刚开始还是扩大规模，我们都会构建和运营值得您信赖的高效养蜂场。</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rehabilitation Plan</t>
+          <t>Environmental Auditing</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>rehabilitation-plan</t>
+          <t>environmental-auditing</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Turn disturbed land into a lasting asset. Our tailored rehabilitation plans restore soils, vegetation and ecosystems to productive, agreed end-uses that satisfy regulators and stakeholders alike. We assess site conditions, design species-appropriate restoration, and set clear success criteria and monitoring. Whether for mining, construction or agriculture, we help you leave land healthier than you found it.</t>
+          <t>Stay ahead of compliance risks. Our independent environmental audits give you an honest, expert picture of how your operations measure up against environmental laws, permit conditions and your own management plans. We identify gaps before regulators do, quantify your risks, and deliver practical, prioritised corrective actions. The result is a stronger licence to operate, fewer surprises, and a demonstrable commitment to environmental responsibility.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>🌱</t>
+          <t>📋</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -3804,41 +3929,81 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H5" t="b">
         <v>1</v>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Ukaguzi wa Mazingira</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Kaa mbele ya hatari za kufuata. Ukaguzi wetu huru wa mazingira hukupa picha ya uaminifu, ya kitaalamu ya jinsi shughuli zako zinavyolingana na sheria za mazingira, masharti ya vibali na mipango yako mwenyewe ya usimamizi. Tunatambua mapengo kabla ya wadhibiti kufanya, kuhesabu hatari zako, na kutoa vitendo vya urekebishaji vilivyopewa kipaumbele. Matokeo yake ni leseni yenye nguvu zaidi ya kufanya kazi, maajabu machache, na kujitolea kuonyeshwa kwa uwajibikaji wa mazingira.</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Audit environnemental</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Gardez une longueur d’avance sur les risques de non-conformité. Nos audits environnementaux indépendants vous donnent une image honnête et experte de la façon dont vos opérations se comparent aux lois environnementales, aux conditions des permis et à vos propres plans de gestion. Nous identifions les lacunes avant les régulateurs, quantifions vos risques et proposons des actions correctives pratiques et hiérarchisées. Le résultat est une licence d’exploitation plus forte, moins de surprises et un engagement démontrable en faveur de la responsabilité environnementale.</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>التدقيق البيئي</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>البقاء في صدارة مخاطر الامتثال. تمنحك عمليات التدقيق البيئي المستقلة لدينا صورة صادقة وخبيرة عن كيفية مقارنة عملياتك بالقوانين البيئية وشروط التصاريح وخطط الإدارة الخاصة بك. نحن نحدد الفجوات قبل قيام الجهات التنظيمية بذلك، ونحدد المخاطر التي تواجهك، ونقدم إجراءات تصحيحية عملية ذات أولوية. والنتيجة هي الحصول على ترخيص أقوى للعمل، ومفاجآت أقل، والتزام واضح بالمسؤولية البيئية.</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Экологический аудит</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Будьте впереди рисков, связанных с соблюдением требований. Наши независимые экологические аудиты дадут вам честную и экспертную картину того, насколько ваша деятельность соответствует экологическим законам, условиям разрешений и вашим собственным планам управления. Мы выявляем пробелы раньше, чем это сделают регулирующие органы, количественно оцениваем ваши риски и реализуем практические, приоритетные корректирующие действия. Результатом является более надежная лицензия на эксплуатацию, меньшее количество сюрпризов и очевидная приверженность экологической ответственности.</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>环境审核</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>领先于合规风险。我们的独立环境审核可以让您诚实、专业地了解您的运营如何符合环境法、许可条件和您自己的管理计划。我们先于监管机构发现差距，量化您的风险，并提供切实可行的、优先的纠正措施。其结果是获得更严格的运营许可、更少的意外以及对环境责任的明显承诺。</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Decommissioning Plan</t>
+          <t>General Workplace Compliance</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>decommissioning-plan</t>
+          <t>workplace-compliance</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Decommission safely and avoid costly surprises. We plan the full, safe shutdown of your facilities — including a thorough environmental performance evaluation — so you meet every closure obligation with zero guesswork. Our plans cover dismantling, waste and contamination management, site restoration and regulatory sign-off. Engage us early and decommission with confidence, control and full compliance.</t>
+          <t>Make compliance effortless. We build the occupational health and safety policies, procedures and inspection systems that keep your workplace safe, audit-ready and fully aligned with the law. From drafting clear policies to running practical inspections and closing gaps, we give you a compliance framework that actually works day to day. Stay on the right side of regulators — and protect your people — with confidence.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>🏗️</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -3846,45 +4011,85 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>environment</t>
+          <t>ohs</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H6" t="b">
         <v>1</v>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Uzingatiaji Mkuu wa Mahali pa Kazi</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Fanya utiifu kuwa rahisi. Tunaunda sera za afya na usalama kazini, taratibu na mifumo ya ukaguzi ambayo huweka eneo lako la kazi salama, tayari kukaguliwa na kupatana kikamilifu na sheria. Kuanzia kuandaa sera zilizo wazi hadi kufanya ukaguzi wa vitendo na kuziba mapengo, tunakupa mfumo wa utiifu ambao hufanya kazi siku hadi siku. Kaa upande wa kulia wa wadhibiti - na ulinde watu wako - kwa ujasiri.</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Conformité générale du lieu de travail</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Assurez la conformité sans effort. Nous élaborons des politiques, des procédures et des systèmes d'inspection en matière de santé et de sécurité au travail qui garantissent la sécurité de votre lieu de travail, sont prêts pour les audits et sont pleinement conformes à la loi. De la rédaction de politiques claires à la réalisation d'inspections pratiques et à la réduction des lacunes, nous vous proposons un cadre de conformité qui fonctionne réellement au quotidien. Restez du bon côté des régulateurs et protégez vos collaborateurs en toute confiance.</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>الامتثال العام في مكان العمل</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>اجعل الامتثال سهلاً. نحن نبني سياسات وإجراءات وأنظمة التفتيش المتعلقة بالصحة والسلامة المهنية التي تحافظ على مكان عملك آمنًا وجاهزًا للتدقيق ومتوافقًا تمامًا مع القانون. بدءًا من صياغة سياسات واضحة وحتى إجراء عمليات التفتيش العملية وسد الثغرات، نقدم لك إطارًا للامتثال يعمل فعليًا يومًا بعد يوم. ابق على الجانب الصحيح من الجهات التنظيمية - واحمِ موظفيك - بثقة.</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Общее соблюдение требований на рабочем месте</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Сделайте соблюдение требований легким. Мы разрабатываем политику, процедуры и системы контроля в области охраны труда и техники безопасности, которые обеспечивают безопасность вашего рабочего места, готовность к аудиту и полное соответствие закону. От разработки четких политик до проведения практических проверок и устранения пробелов — мы предоставляем вам систему обеспечения соответствия, которая действительно работает изо дня в день. Оставайтесь на правильной стороне регулирующих органов и защищайте своих людей с уверенностью.</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>一般工作场所合规性</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>让合规变得毫不费力。我们制定职业健康和安全政策、程序和检查系统，确保您的工作场所安全、做好审计准备并完全符合法律。从起草明确的政策到进行实际检查和缩小差距，我们为您提供了一个日常有效的合规框架。充满信心地站在监管机构的正确一边，并保护您的员工。</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Engineering Design</t>
+          <t>Beekeeping Equipment &amp; Inputs</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>engineering-design</t>
+          <t>beekeeping-equipment-inputs</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Engineer your waste and water infrastructure right the first time. We provide environmental engineering design for the structures that keep your operation safe and compliant — Tailings Storage Facility (TSF), Waste Rock Dump (WRD), Drainage, Waste Storage Facility (WSF), Waste Stockpile (WSP) and Landfill. Our designs balance safety, regulatory compliance and cost-effectiveness, backed by sound geotechnical and hydrological analysis. Build with a partner who gets the engineering — and the environment — right.</t>
+          <t>Everything you need to succeed, from one trusted supplier. We provide quality Langstroth and top-bar beehives, protective gear, hive tools, healthy bee colonies, queen bees and harvesting equipment. Start strong and stay productive with dependable inputs sourced and supported by experts who understand beekeeping.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>📐</t>
+          <t>🧰</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -3892,45 +4097,85 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>environment</t>
+          <t>beekeeping</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H7" t="b">
         <v>1</v>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Vifaa na Pembejeo za Ufugaji Nyuki</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Kila kitu unachohitaji ili kufanikiwa, kutoka kwa muuzaji mmoja anayeaminika. Tunatoa mizinga ya ubora wa Langstroth na upau wa juu, zana za kinga, zana za mizinga, makundi ya nyuki wenye afya nzuri, malkia wa nyuki na vifaa vya kuvuna. Anza kwa nguvu na uendelee kuwa na tija kwa pembejeo zinazotegemewa zinazopatikana na kuungwa mkono na wataalam wanaoelewa ufugaji nyuki.</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Équipements et intrants apicoles</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Tout ce dont vous avez besoin pour réussir, auprès d'un seul fournisseur de confiance. Nous fournissons des ruches Langstroth et Top-Bar de qualité, des équipements de protection, des outils de ruche, des colonies d'abeilles saines, des reines des abeilles et du matériel de récolte. Commencez fort et restez productif avec des intrants fiables provenant et soutenus par des experts qui comprennent l’apiculture.</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>معدات ومدخلات تربية النحل</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>كل ما تحتاجه لتحقيق النجاح، من مورد واحد موثوق به. نحن نقدم خلايا لانجستروث وخلايا النحل ذات الجودة العالية، ومعدات الحماية، وأدوات الخلية، ومستعمرات النحل الصحية، وملكة النحل، ومعدات الحصاد. ابدأ بقوة وحافظ على إنتاجيتك باستخدام مدخلات يمكن الاعتماد عليها يتم الحصول عليها ودعمها من خبراء يفهمون تربية النحل.</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Оборудование и материалы для пчеловодства</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Все, что вам нужно для успеха, от одного проверенного поставщика. Мы предоставляем качественные ульи Лангстрота и ульи с верхней перекладиной, защитное снаряжение, инструменты для ульев, здоровые пчелиные семьи, пчелиные матки и оборудование для сбора урожая. Начните уверенно и оставайтесь продуктивными, используя надежные материалы, полученные и поддерживаемые экспертами, разбирающимися в пчеловодстве.</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>养蜂设备和投入</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>您成功所需的一切均来自值得信赖的供应商。我们提供优质的 Langstroth 和顶栏蜂箱、防护装备、蜂巢工具、健康的蜂群、蜂王和收获设备。依靠了解养蜂业的专家提供的可靠投入和支持，开始强劲并保持生产力。</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Feasibility Studies</t>
+          <t>Mine Closure &amp; Rehabilitation Plan</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>feasibility-studies</t>
+          <t>mine-closure-rehabilitation</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Invest with certainty. Our technical and environmental feasibility studies for mining and agricultural projects give you the clear, bankable insight you need before committing resources. We evaluate technical viability, environmental constraints, costs and risks, and present findings that stand up to investors and lenders. Make your next decision on solid ground, with analysis you can trust.</t>
+          <t>Close responsibly and protect your legacy. We design practical, regulator-approved mine closure and rehabilitation plans that meet your legal obligations while restoring land the community can trust. Our team addresses landform design, revegetation, water management and post-closure monitoring, with realistic cost estimates you can plan around. Start planning early with us and turn closure from a liability into a well-managed, credible commitment.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>📊</t>
+          <t>⛏️</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -3942,36 +4187,76 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H8" t="b">
         <v>1</v>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Mpango wa Kufunga &amp; Ukarabati wa Migodi</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Funga kwa kuwajibika na ulinde urithi wako. Tunabuni mipango ya vitendo, iliyoidhinishwa na udhibiti wa kufungwa na ukarabati wa migodi ambayo inakidhi majukumu yako ya kisheria huku tukirejesha ardhi ambayo jumuiya inaweza kuamini. Timu yetu inashughulikia muundo wa ardhi, upandaji miti, usimamizi wa maji na ufuatiliaji wa baada ya kufungwa, na makadirio ya gharama halisi ambayo unaweza kupanga karibu. Anza kupanga mapema nasi na ugeuze kufungwa kutoka kwa dhima hadi dhamira inayodhibitiwa vyema na inayoaminika.</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Plan de fermeture et de réhabilitation de la mine</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Fermez de manière responsable et protégez votre héritage. Nous concevons des plans pratiques de fermeture de mine et de réhabilitation approuvés par les régulateurs qui répondent à vos obligations légales tout en restaurant des terres auxquelles la communauté peut avoir confiance. Notre équipe s'occupe de la conception du relief, de la revégétalisation, de la gestion de l'eau et de la surveillance post-fermeture, avec des estimations de coûts réalistes que vous pouvez planifier. Commencez à planifier tôt avec nous et transformez la clôture d’un passif en un engagement crédible et bien géré.</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>خطة إغلاق المناجم وإعادة تأهيلها</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>إغلاق بمسؤولية وحماية تراثك. نحن نصمم خططًا عملية لإغلاق المناجم وإعادة تأهيلها ومعتمدة من قبل الجهات التنظيمية والتي تلبي التزاماتك القانونية مع استعادة الأراضي التي يمكن للمجتمع أن يثق بها. يعالج فريقنا تصميم التضاريس وإعادة الغطاء النباتي وإدارة المياه ومراقبة ما بعد الإغلاق، مع تقديرات تكلفة واقعية يمكنك التخطيط لها. ابدأ التخطيط مبكرًا معنا وحوّل إغلاق المسؤولية إلى التزام موثوق به ومُدار بشكل جيد.</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>План закрытия и реабилитации шахты</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Закройте ответственно и защитите свое наследие. Мы разрабатываем практичные, одобренные регулирующими органами планы закрытия и реабилитации шахт, которые соответствуют вашим юридическим обязательствам и одновременно восстанавливают земли, которым может доверять сообщество. Наша команда занимается проектированием ландшафта, восстановлением растительности, управлением водными ресурсами и мониторингом после закрытия, предоставляя реалистичные оценки затрат, которые вы можете спланировать. Начните планировать вместе с нами заранее и превратите закрытие из обязательства в хорошо управляемое и заслуживающее доверия обязательство.</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>矿山关闭及恢复计划</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>负责任地关闭并保护您的遗产。我们设计实用的、经监管机构批准的矿山关闭和恢复计划，以满足您的法律义务，同时恢复社区可以信任的土地。我们的团队致力于地形设计、植被恢复、水资源管理和关闭后监测，并提供实际的成本估算，供您规划。尽早与我们一起开始计划，将关闭从一项责任转变为管理良好、可信的承诺。</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Training on Environmental Management</t>
+          <t>Training on OHS Issues</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>environmental-management-training</t>
+          <t>ohs-training</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Empower your team to manage compliance in-house. Our hands-on environmental management training builds lasting capacity that reduces risk and saves you money year after year. We deliver practical, workplace-relevant sessions on regulatory requirements, monitoring, reporting and best practice — tailored to your operation. Invest in your people and turn environmental management into a core strength.</t>
+          <t>Build a safety-first culture that lasts. Our practical occupational health and safety training equips your workforce to work safely, cut downtime and meet every regulatory expectation. We deliver engaging, workplace-relevant sessions — from hazard awareness to emergency response — tailored to your industry and risks. Turn safety from a checkbox into a genuine, lasting culture.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -3984,45 +4269,85 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>environment</t>
+          <t>ohs</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H9" t="b">
         <v>1</v>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Mafunzo juu ya Masuala ya OHS</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Jenga utamaduni wa usalama-kwanza unaodumu. Mafunzo yetu ya vitendo ya afya na usalama kazini huwezesha wafanyikazi wako kufanya kazi kwa usalama, kupunguza muda wa kupumzika na kukidhi kila matarajio ya udhibiti. Tunatoa vipindi vinavyohusika, vinavyohusiana na mahali pa kazi - kutoka kwa uhamasishaji wa hatari hadi jibu la dharura - vinavyolenga sekta yako na hatari. Geuza usalama kutoka kwa kisanduku cha kuteua kuwa utamaduni halisi na wa kudumu.</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Formation sur les questions de SST</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Construisez une culture axée sur la sécurité qui dure. Notre formation pratique en matière de santé et de sécurité au travail permet à votre personnel de travailler en toute sécurité, de réduire les temps d'arrêt et de répondre à toutes les attentes réglementaires. Nous proposons des sessions engageantes et pertinentes sur le lieu de travail – de la sensibilisation aux dangers à l’intervention d’urgence – adaptées à votre secteur et à vos risques. Transformez la sécurité d’une simple case à cocher en une véritable culture durable.</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>التدريب على قضايا الصحة والسلامة المهنية</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>بناء ثقافة السلامة أولاً التي تدوم. يعمل تدريبنا العملي في مجال الصحة والسلامة المهنية على تجهيز القوى العاملة لديك للعمل بأمان وتقليل وقت التوقف عن العمل وتلبية كل التوقعات التنظيمية. نحن نقدم جلسات جذابة وذات صلة بمكان العمل - بدءًا من الوعي بالمخاطر وحتى الاستجابة لحالات الطوارئ - ومصممة خصيصًا لتناسب صناعتك والمخاطر التي تواجهها. قم بتحويل الأمان من مربع الاختيار إلى ثقافة حقيقية ودائمة.</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Обучение по вопросам охраны труда</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Создайте устойчивую культуру, в которой безопасность превыше всего. Наше практическое обучение по охране труда и технике безопасности поможет вашим сотрудникам работать безопасно, сократить время простоев и соответствовать всем нормативным требованиям. Мы проводим увлекательные занятия, актуальные для рабочего места — от информирования об опасностях до реагирования на чрезвычайные ситуации — с учетом вашей отрасли и рисков. Превратите безопасность из флажка в подлинную, прочную культуру.</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>职业健康安全问题培训</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>建立持久的安全第一文化。我们实用的职业健康和安全培训使您的员工能够安全工作、减少停机时间并满足每项监管期望。我们提供引人入胜的、与工作场所相关的课程——从危险意识到应急响应——根据您的行业和风险量身定制。将安全从复选框转变为真正、持久的文化。</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Risk Assessment</t>
+          <t>Honey &amp; Bee Products Processing</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>risk-assessment</t>
+          <t>honey-bee-products-processing</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Protect your people and your productivity. Our thorough workplace risk assessments uncover hidden hazards and deliver practical controls that prevent incidents before they happen. We systematically identify, evaluate and prioritise risks across your operations, then recommend cost-effective measures that keep workers safe and operations running. Reduce accidents, lower costs, and demonstrate genuine care for your workforce.</t>
+          <t>Turn your harvest into premium, market-ready products. Our honey harvesting, extraction, filtration, packaging and value-added processing help you meet quality standards and command better prices. From raw comb to beautifully packaged, branded honey and bee products, we help you add value at every step.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>⚠️</t>
+          <t>🍯</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -4030,45 +4355,85 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>ohs</t>
+          <t>beekeeping</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H10" t="b">
         <v>1</v>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Usindikaji wa Bidhaa za Asali na Nyuki</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Geuza mavuno yako kuwa bidhaa bora, zilizo tayari sokoni. Uvunaji wetu wa asali, uchimbaji, uchujaji, ufungaji na usindikaji wa ongezeko la thamani hukusaidia kufikia viwango vya ubora na kuagiza bei bora. Kuanzia sega mbichi hadi asali iliyofungashwa vizuri, yenye chapa na bidhaa za nyuki, tunakusaidia kuongeza thamani katika kila hatua.</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Transformation du miel et des produits apicoles</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Transformez votre récolte en produits haut de gamme prêts à être commercialisés. Nos activités de récolte, d’extraction, de filtration, d’emballage et de transformation à valeur ajoutée du miel vous aident à respecter les normes de qualité et à obtenir de meilleurs prix. Du rayon brut au miel et aux produits apicoles de marque joliment emballés, nous vous aidons à ajouter de la valeur à chaque étape.</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>تصنيع منتجات العسل والنحل</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>حول محصولك إلى منتجات متميزة وجاهزة للسوق. يساعدك حصاد العسل واستخراجه وترشيحه وتعبئته ومعالجته ذات القيمة المضافة على تلبية معايير الجودة والحصول على أسعار أفضل. بدءًا من المشط الخام وحتى منتجات العسل والنحل المعبأة بشكل جميل وذات العلامات التجارية، نساعدك على إضافة قيمة في كل خطوة.</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Переработка меда и продуктов пчеловодства</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Превратите свой урожай в продукцию премиум-класса, готовую к продаже. Наш сбор, экстракция, фильтрация, упаковка и обработка меда с добавленной стоимостью помогают вам соответствовать стандартам качества и предлагать более выгодные цены. От сырых сотов до красиво упакованного фирменного меда и продуктов пчеловодства — мы помогаем вам повышать ценность на каждом этапе.</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>蜂蜜及蜂产品加工</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>将您的收获转化为优质、可上市的产品。我们的蜂蜜采收、提取、过滤、包装和增值加工可帮助您满足质量标准并获得更优惠的价格。从原蜂巢到包装精美的品牌蜂蜜和蜂产品，我们在每一步都帮助您增加价值。</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>General Workplace Compliance</t>
+          <t>Rehabilitation Plan</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>workplace-compliance</t>
+          <t>rehabilitation-plan</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Make compliance effortless. We build the occupational health and safety policies, procedures and inspection systems that keep your workplace safe, audit-ready and fully aligned with the law. From drafting clear policies to running practical inspections and closing gaps, we give you a compliance framework that actually works day to day. Stay on the right side of regulators — and protect your people — with confidence.</t>
+          <t>Turn disturbed land into a lasting asset. Our tailored rehabilitation plans restore soils, vegetation and ecosystems to productive, agreed end-uses that satisfy regulators and stakeholders alike. We assess site conditions, design species-appropriate restoration, and set clear success criteria and monitoring. Whether for mining, construction or agriculture, we help you leave land healthier than you found it.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>🌱</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -4076,40 +4441,80 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>ohs</t>
+          <t>environment</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H11" t="b">
         <v>1</v>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Mpango wa Ukarabati</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Badilisha ardhi iliyovurugwa kuwa mali ya kudumu. Mipango yetu ya urekebishaji iliyoundwa inarejesha udongo, mimea na mifumo ikolojia kwa matumizi yenye tija, yaliyokubaliwa ambayo yanakidhi wadhibiti na washikadau sawa. Tunatathmini hali ya tovuti, kuunda urejeshaji unaofaa wa spishi, na kuweka wazi vigezo vya mafanikio na ufuatiliaji. Iwe kwa madini, ujenzi au kilimo, tunakusaidia kuacha ardhi ikiwa na afya kuliko ulivyoipata.</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Plan de réhabilitation</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Transformez les terres perturbées en un atout durable. Nos plans de réhabilitation sur mesure restaurent les sols, la végétation et les écosystèmes vers des utilisations finales productives et convenues qui satisfont à la fois les régulateurs et les parties prenantes. Nous évaluons les conditions du site, concevons une restauration adaptée aux espèces et établissons des critères de réussite et de surveillance clairs. Que ce soit pour l’exploitation minière, la construction ou l’agriculture, nous vous aidons à laisser la terre plus saine que vous ne l’avez trouvée.</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>خطة إعادة التأهيل</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>تحويل الأراضي المضطربة إلى أصول دائمة. تعمل خطط إعادة التأهيل المصممة خصيصًا لدينا على إعادة التربة والغطاء النباتي والنظم البيئية إلى استخدامات نهائية منتجة ومتفق عليها ترضي الجهات التنظيمية وأصحاب المصلحة على حدٍ سواء. نقوم بتقييم ظروف الموقع، وتصميم عمليات الاستعادة المناسبة للأنواع، ووضع معايير نجاح ورصد واضحة. سواء كان الأمر يتعلق بالتعدين أو البناء أو الزراعة، فإننا نساعدك على ترك الأرض أكثر صحة مما وجدتها عليه.</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>План реабилитации</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Превратите нарушенную землю в долгосрочный актив. Наши индивидуальные планы реабилитации восстанавливают почвы, растительность и экосистемы до продуктивного, согласованного конечного использования, которое удовлетворяет как регулирующие органы, так и заинтересованные стороны. Мы оцениваем состояние участка, проектируем восстановление с учетом видов и устанавливаем четкие критерии успеха и мониторинг. Будь то горнодобывающая промышленность, строительство или сельское хозяйство, мы помогаем вам оставить землю более здоровой, чем вы ее видели.</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>康复计划</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>将受干扰的土地变成持久的资产。我们量身定制的恢复计划可将土壤、植被和生态系统恢复到生产性的、商定的最终用途，从而满足监管机构和利益相关者的要求。我们评估场地条件，设计适合物种的恢复，并设定明确的成功标准和监控。无论是采矿、建筑还是农业，我们都能帮助您让土地变得比发现时更健康。</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Training on OHS Issues</t>
+          <t>Training &amp; Consultancy</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ohs-training</t>
+          <t>beekeeping-training-consultancy</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Build a safety-first culture that lasts. Our practical occupational health and safety training equips your workforce to work safely, cut downtime and meet every regulatory expectation. We deliver engaging, workplace-relevant sessions — from hazard awareness to emergency response — tailored to your industry and risks. Turn safety from a checkbox into a genuine, lasting culture.</t>
+          <t>Build a profitable beekeeping enterprise with expert guidance. From practical training and capacity building to feasibility studies, business planning and certification support, we give you the knowledge and confidence to succeed. Whether you are a smallholder or an investor, we help you turn beekeeping into a thriving, bankable business.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -4122,45 +4527,85 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>ohs</t>
+          <t>beekeeping</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H12" t="b">
         <v>1</v>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Mafunzo na Ushauri</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Jenga biashara ya ufugaji nyuki yenye faida kwa mwongozo wa kitaalam. Kuanzia mafunzo ya vitendo na kujenga uwezo hadi upembuzi yakinifu, upangaji biashara na usaidizi wa uidhinishaji, tunakupa maarifa na ujasiri wa kufaulu. Iwe wewe ni mfanyabiashara mdogo au mwekezaji, tunakusaidia kugeuza ufugaji nyuki kuwa biashara inayostawi, inayoweza kulipwa.</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Formation et conseil</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Créez une entreprise apicole rentable avec les conseils d’experts. De la formation pratique et du renforcement des capacités aux études de faisabilité, en passant par la planification commerciale et l'assistance à la certification, nous vous donnons les connaissances et la confiance nécessaires pour réussir. Que vous soyez un petit exploitant ou un investisseur, nous vous aidons à transformer l’apiculture en une entreprise florissante et rentable.</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>التدريب والاستشارات</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>بناء مؤسسة مربحة لتربية النحل بتوجيه من الخبراء. بدءًا من التدريب العملي وبناء القدرات وحتى دراسات الجدوى وتخطيط الأعمال ودعم الشهادات، نقدم لك المعرفة والثقة لتحقيق النجاح. سواء كنت من أصحاب الحيازات الصغيرة أو مستثمرًا، فإننا نساعدك على تحويل تربية النحل إلى عمل مزدهر وقابل للتمويل.</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Обучение и консультации</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Постройте прибыльное пчеловодческое предприятие под руководством экспертов. От практического обучения и наращивания потенциала до технико-экономических обоснований, бизнес-планирования и поддержки в сертификации — мы даем вам знания и уверенность в успехе. Независимо от того, являетесь ли вы мелким землевладельцем или инвестором, мы поможем вам превратить пчеловодство в процветающий прибыльный бизнес.</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>培训与咨询</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>在专家指导下建立盈利的养蜂企业。从实践培训和能力建设到可行性研究、业务规划和认证支持，我们为您提供成功的知识和信心。无论您是小农还是投资者，我们都可以帮助您将养蜂业变成一项蓬勃发展、可盈利的业务。</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Apiary Establishment &amp; Management</t>
+          <t>Decommissioning Plan</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>apiary-establishment-management</t>
+          <t>decommissioning-plan</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Start your apiary the right way and keep it thriving. We handle everything from expert site selection and hive installation to colony management, pest and disease control, and ongoing maintenance — so your bees stay healthy and your harvests stay strong, season after season. Whether you are starting fresh or scaling up, we build and run productive apiaries you can rely on.</t>
+          <t>Decommission safely and avoid costly surprises. We plan the full, safe shutdown of your facilities — including a thorough environmental performance evaluation — so you meet every closure obligation with zero guesswork. Our plans cover dismantling, waste and contamination management, site restoration and regulatory sign-off. Engage us early and decommission with confidence, control and full compliance.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>🐝</t>
+          <t>🏗️</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -4168,45 +4613,85 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>beekeeping</t>
+          <t>environment</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H13" t="b">
         <v>1</v>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Mpango wa Kufuta</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Ondoa kwa usalama na uepuke mshangao wa gharama kubwa. Tunapanga kuzima kabisa na kwa usalama kwa vifaa vyako - ikiwa ni pamoja na tathmini ya kina ya utendakazi wa mazingira - ili utimize kila dhima ya kufungwa bila kubahatisha. Mipango yetu inashughulikia uvunjaji, udhibiti wa taka na uchafuzi, urejeshaji wa tovuti na uondoaji wa udhibiti. Tushirikishe mapema na usitishe kazi kwa kujiamini, udhibiti na kufuata kikamilifu.</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Plan de déclassement</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Mettez hors service en toute sécurité et évitez les surprises coûteuses. Nous planifions la fermeture complète et sûre de vos installations, y compris une évaluation approfondie des performances environnementales, afin que vous respectiez chaque obligation de fermeture sans aucune hypothèse. Nos plans couvrent le démantèlement, la gestion des déchets et de la contamination, la restauration du site et l'approbation réglementaire. Engagez-nous rapidement et mettez hors service en toute confiance, contrôle et conformité totale.</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>خطة التفكيك</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>الخروج من الخدمة بأمان وتجنب المفاجآت المكلفة. نحن نخطط للإغلاق الكامل والآمن لمنشآتك - بما في ذلك تقييم شامل للأداء البيئي - حتى تتمكن من الوفاء بكل التزامات الإغلاق دون أي تخمين. تغطي خططنا التفكيك وإدارة النفايات والتلوث وترميم الموقع والتوقيع التنظيمي. أشركنا مبكرًا وخرج من الخدمة بثقة وتحكم وامتثال كامل.</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>План вывода из эксплуатации</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Безопасный вывод из эксплуатации и избежание дорогостоящих сюрпризов. Мы планируем полное и безопасное закрытие ваших объектов, включая тщательную оценку экологических показателей, чтобы вы выполнили все обязательства по закрытию без каких-либо догадок. В наши планы входит демонтаж, управление отходами и загрязнениями, восстановление объектов и согласование нормативных требований. Привлеките нас заранее и выведите из эксплуатации с уверенностью, контролем и полным соблюдением требований.</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>退役计划</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>安全退役并避免代价高昂的意外情况。我们计划全面、安全地关闭您的设施，包括彻底的环境绩效评估，以便您零猜测地履行每一项关闭义务。我们的计划涵盖拆除、废物和污染管理、场地恢复和监管批准。尽早与我们合作并充满信心、控制力和完全合规地退役。</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Beekeeping Equipment &amp; Inputs</t>
+          <t>Engineering Design</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>beekeeping-equipment-inputs</t>
+          <t>engineering-design</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Everything you need to succeed, from one trusted supplier. We provide quality Langstroth and top-bar beehives, protective gear, hive tools, healthy bee colonies, queen bees and harvesting equipment. Start strong and stay productive with dependable inputs sourced and supported by experts who understand beekeeping.</t>
+          <t>Engineer your waste and water infrastructure right the first time. We provide environmental engineering design for the structures that keep your operation safe and compliant — Tailings Storage Facility (TSF), Waste Rock Dump (WRD), Drainage, Waste Storage Facility (WSF), Waste Stockpile (WSP) and Landfill. Our designs balance safety, regulatory compliance and cost-effectiveness, backed by sound geotechnical and hydrological analysis. Build with a partner who gets the engineering — and the environment — right.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>🧰</t>
+          <t>📐</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -4214,45 +4699,85 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>beekeeping</t>
+          <t>environment</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H14" t="b">
         <v>1</v>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Ubunifu wa Uhandisi</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Tengeneza miundombinu yako ya taka na maji mara ya kwanza. Tunatoa usanifu wa uhandisi wa mazingira kwa miundo inayoweka utendakazi wako salama na utiifu - Kituo cha Kuhifadhi Tailings (TSF), Dampo la Mawe Machafu (WRD), Mifereji ya Maji, Kituo cha Kuhifadhi Taka (WSF), Rundo la Taka (WSP) na Jalada. Miundo yetu inasawazisha usalama, utiifu wa udhibiti na ufaafu wa gharama, unaoungwa mkono na uchanganuzi mzuri wa kijiotekiniki na kihaidrolojia. Jenga na mshirika ambaye anapata uhandisi - na mazingira - sawa.</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Conception technique</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Concevez correctement votre infrastructure de gestion des déchets et de l'eau du premier coup. Nous fournissons une conception technique environnementale pour les structures qui assurent la sécurité et la conformité de vos opérations : installation de stockage de résidus (TSF), décharge de stériles (WRD), drainage, installation de stockage de déchets (WSF), tas de déchets (WSP) et décharge. Nos conceptions équilibrent sécurité, conformité réglementaire et rentabilité, soutenues par des analyses géotechniques et hydrologiques solides. Construisez avec un partenaire qui maîtrise l’ingénierie – et l’environnement – ​​correctement.</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>التصميم الهندسي</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>قم بتصميم البنية التحتية للنفايات والمياه الخاصة بك بشكل صحيح من المرة الأولى. نحن نقدم تصميمًا هندسيًا بيئيًا للهياكل التي تحافظ على أمان عملياتك وامتثالها - مرافق تخزين المخلفات (TSF)، ومكب النفايات الصخرية (WRD)، والصرف الصحي، ومرافق تخزين النفايات (WSF)، ومخزون النفايات (WSP)، ومكب النفايات. تعمل تصميماتنا على تحقيق التوازن بين السلامة والامتثال التنظيمي وفعالية التكلفة، مدعومة بالتحليل الجيوتقني والهيدرولوجي السليم. قم بالبناء مع شريك يتقن الهندسة - والبيئة - بشكل صحيح.</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Инженерное проектирование</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Спроектируйте инфраструктуру отходов и водоснабжения правильно с первого раза. Мы обеспечиваем экологическое инженерное проектирование сооружений, которые обеспечивают безопасность и соответствие требованиям вашей деятельности — хвостохранилище (ХХ), отвал пустой породы (WRD), дренаж, хранилище отходов (WSF), склад отходов (WSP) и полигон. Наши проекты сочетают в себе безопасность, соответствие нормативным требованиям и экономическую эффективность, подкрепленные тщательным геотехническим и гидрологическим анализом. Стройте вместе с партнером, который правильно разбирается в проектировании и окружающей среде.</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>工程设计</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>第一次就正确设计您的废物和水基础设施。我们为确保您的运营安全和合规的结构提供环境工程设计 - 尾矿储存设施 (TSF)、废石堆 (WRD)、排水、废物储存设施 (WSF)、废物储存设施 (WSP) 和垃圾填埋场。我们的设计以可靠的岩土工程和水文分析为支持，平衡了安全性、法规遵从性和成本效益。与正确设计和环境的合作伙伴一起构建。</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Honey &amp; Bee Products Processing</t>
+          <t>Feasibility Studies</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>honey-bee-products-processing</t>
+          <t>feasibility-studies</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Turn your harvest into premium, market-ready products. Our honey harvesting, extraction, filtration, packaging and value-added processing help you meet quality standards and command better prices. From raw comb to beautifully packaged, branded honey and bee products, we help you add value at every step.</t>
+          <t>Invest with certainty. Our technical and environmental feasibility studies for mining and agricultural projects give you the clear, bankable insight you need before committing resources. We evaluate technical viability, environmental constraints, costs and risks, and present findings that stand up to investors and lenders. Make your next decision on solid ground, with analysis you can trust.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>🍯</t>
+          <t>📊</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -4260,71 +4785,65 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>beekeeping</t>
+          <t>environment</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H15" t="b">
         <v>1</v>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Training &amp; Consultancy</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>beekeeping-training-consultancy</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Build a profitable beekeeping enterprise with expert guidance. From practical training and capacity building to feasibility studies, business planning and certification support, we give you the knowledge and confidence to succeed. Whether you are a smallholder or an investor, we help you turn beekeeping into a thriving, bankable business.</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>🎓</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>beekeeping</t>
-        </is>
-      </c>
-      <c r="G16" t="n">
-        <v>4</v>
-      </c>
-      <c r="H16" t="b">
-        <v>1</v>
-      </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Upembuzi Yakinifu</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Wekeza kwa uhakika. Tafiti zetu za upembuzi yakinifu wa kiufundi na kimazingira kwa ajili ya miradi ya madini na kilimo hukupa ufahamu wazi, unaoweza kulipwa unaohitaji kabla ya kutoa rasilimali. Tunatathmini uwezekano wa kiufundi, vikwazo vya mazingira, gharama na hatari, na kuwasilisha matokeo ambayo yanalingana na wawekezaji na wakopeshaji. Fanya uamuzi wako unaofuata kwa msingi thabiti, na uchanganuzi unaoweza kuamini.</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Études de faisabilité</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Investissez avec certitude. Nos études de faisabilité technique et environnementale de projets miniers et agricoles vous donnent l’éclairage clair et bancable dont vous avez besoin avant d’engager des ressources. Nous évaluons la viabilité technique, les contraintes environnementales, les coûts et les risques, et présentons des conclusions qui résistent aux investisseurs et aux prêteurs. Prenez votre prochaine décision sur des bases solides, avec une analyse à laquelle vous pouvez faire confiance.</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>دراسات الجدوى</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>استثمر بثقة. تمنحك دراسات الجدوى الفنية والبيئية الخاصة بمشاريع التعدين والزراعة الرؤية الواضحة والمقبولة التي تحتاجها قبل الالتزام بالموارد. نقوم بتقييم الجدوى الفنية، والقيود البيئية، والتكاليف والمخاطر، وتقديم النتائج التي تقف في وجه المستثمرين والمقرضين. اتخذ قرارك التالي على أرض صلبة، مع التحليل الذي يمكنك الوثوق به.</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Технико-экономические исследования</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Инвестируйте с уверенностью. Наши технические и экологические технико-экономические обоснования проектов в горнодобывающей промышленности и сельском хозяйстве дадут вам четкое и ценное представление, необходимое перед выделением ресурсов. Мы оцениваем техническую жизнеспособность, экологические ограничения, затраты и риски и представляем результаты, которые будут полезны инвесторам и кредиторам. Примите следующее решение, опираясь на твердую почву и анализ, которому можно доверять.</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>可行性研究</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>投资有把握。我们针对采矿和农业项目的技术和环境可行性研究为您提供在投入资源之前所需的清晰、可靠的见解。我们评估技术可行性、环境限制、成本和风险，并提出对投资者和贷方经得起考验的调查结果。通过可靠的分析，做出下一个决定。</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4833,7 +5352,11 @@
           <t>500g</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N2" t="inlineStr">
         <is>
           <t>Pure natural honey</t>
@@ -4925,7 +5448,11 @@
           <t>1kg</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N3" t="inlineStr">
         <is>
           <t>Pure natural honey</t>
@@ -5017,7 +5544,11 @@
           <t>500g</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N4" t="inlineStr">
         <is>
           <t>Organic forest honey</t>
@@ -5107,7 +5638,11 @@
           <t>500g</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N5" t="inlineStr">
         <is>
           <t>Acacia honey</t>
@@ -5197,7 +5732,11 @@
           <t>250g</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N6" t="inlineStr">
         <is>
           <t>Pure natural beeswax</t>
@@ -5289,7 +5828,11 @@
           <t>1kg</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N7" t="inlineStr">
         <is>
           <t>Pure natural beeswax</t>
@@ -5473,7 +6016,11 @@
           <t>5kg</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N9" t="inlineStr">
         <is>
           <t>Protective suit, gloves, smoker, hive tool, bee brush, guide book</t>
@@ -5937,7 +6484,11 @@
           <t>5kg</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N14" t="inlineStr">
         <is>
           <t>Includes laying queen, worker bees, brood, honey, and pollen</t>
@@ -6023,7 +6574,11 @@
           <t>0.05kg</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N15" t="inlineStr">
         <is>
           <t>Mated queen bee with 5-8 attendant workers</t>
@@ -6573,7 +7128,11 @@
           <t>30ml</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N21" t="inlineStr">
         <is>
           <t>Bee propolis extract in alcohol base</t>
@@ -6895,7 +7454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7014,29 +7573,6 @@
         <v>4</v>
       </c>
       <c r="E5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Construction</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>construction</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Construction and infrastructure projects</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>5</v>
-      </c>
-      <c r="E6" t="b">
         <v>1</v>
       </c>
     </row>
@@ -7051,7 +7587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB8"/>
+  <dimension ref="A1:AB10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7199,27 +7735,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Modern Apiary Setup for Cooperative</t>
+          <t>SEN WO COMPANY LIMITED IN GEITA REGION</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>modern-apiary-cooperative</t>
+          <t>sen-wo-company-limited-in-geita-region</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Designed and installed 500 modern Langstroth beehives for a farmers cooperative in Dodoma, increasing honey production by 60%.</t>
+          <t>Fee-vert Solution Limited provided comprehensive environmental, engineering, and regulatory compliance services to SEN WO Company Limited in the Geita Region, including the preparation and successful approval of the Environmental and Social Impact Assessment (ESIA), Tailings Storage Facility (TSF) Design approved by the Mining Commission, workplace compliance services including OSHA registration and certification, Fire Permit compliance, and chemical management compliance and permitting through GCLA. These services supported the client in meeting statutory requirements and maintaining safe, environmentally responsible, and compliant mining operations.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>beekeeping</t>
+          <t>environment</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Dodoma Farmers Cooperative</t>
+          <t>SEN WO COMPANY LIMITED IN GEITA REGION</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -7227,125 +7763,53 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Low honey production using traditional hives</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Installed modern Langstroth hives with training</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>60% increase in honey production, 200 farmers trained</t>
-        </is>
-      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="b">
         <v>1</v>
       </c>
       <c r="K2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L2" t="b">
         <v>1</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>media/project_covers/langstroth_beehive_jcryl6</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Uanzishwaji wa Banda la Kisasa la Nyuki kwa Chama cha Ushirika</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Tulibuni na kufunga mizinga 500 ya kisasa ya Langstroth kwa chama cha ushirika cha wakulima huko Dodoma, na kuongeza uzalishaji wa asali kwa asilimia 60.</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Chama cha Ushirika cha Wakulima wa Dodoma</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>Installation d'un Rucher Moderne pour une Coopérative</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Conception et installation de 500 ruches Langstroth modernes pour une coopérative d'agriculteurs à Dodoma, augmentant la production de miel de 60 %.</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>Coopérative des Agriculteurs de Dodoma</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>إنشاء منحل حديث لتعاونية</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>صممنا وركّبنا 500 خلية لانغستروث حديثة لتعاونية مزارعين في دودوما، مما أدى إلى زيادة إنتاج العسل بنسبة 60٪.</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>تعاونية مزارعي دودوما</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>Создание Современной Пасеки для Кооператива</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>Спроектировали и установили 500 современных ульев Лангстрота для фермерского кооператива в Додоме, увеличив производство мёда на 60%.</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>Фермерский кооператив Додомы</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>为合作社建立现代化蜂场</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>为多多马的一个农民合作社设计并安装了500个现代朗氏蜂箱，使蜂蜜产量提高了60%。</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>多多马农民合作社</t>
-        </is>
-      </c>
+          <t>media/project_covers/WhatsApp_Image_2026-07-04_at_14.32.00_1_abutmu</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>EIA for Mining Project</t>
+          <t>SYNERGY TANZANIA CO. LIMITED</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>eia-mining-project</t>
+          <t>synergy-tanzania-co-limited</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Conducted comprehensive Environmental Impact Assessment for a large-scale mining project in Geita region.</t>
+          <t>Fee-vert provided comprehensive environmental, engineering, and regulatory compliance services to Synergy Tanzania Co. Limited, including the preparation and successful approval of the Environmental and Social Impact Assessment (ESIA), Tailings Storage Facility (TSF) Design approved by the Mining Commission, and workplace compliance services, including OSHA registration and certification, supporting the client in achieving regulatory compliance and responsible mining operations.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -7355,7 +7819,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Geita Gold Mining Ltd</t>
+          <t>SYNERGY TANZANIA CO. LIMITED</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -7363,135 +7827,64 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Complex regulatory requirements and community concerns</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Full ESIA with extensive stakeholder engagement</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>NEMC approval obtained, community agreement signed</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="b">
         <v>1</v>
       </c>
       <c r="K3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L3" t="b">
         <v>1</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>media/project_covers/GRAPHITE_MINING_PROJECT_lkomdi</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>EIA kwa Mradi wa Uchimbaji Madini</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Tulifanya Tathmini kamili ya Athari za Kimazingira kwa mradi mkubwa wa uchimbaji madini mkoani Geita.</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Geita Gold Mining Ltd</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>EIE pour un Projet Minier</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Réalisation d'une Étude d'Impact Environnemental complète pour un projet minier à grande échelle dans la région de Geita.</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>Geita Gold Mining Ltd</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>تقييم الأثر البيئي لمشروع تعديني</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>أجرينا تقييمًا شاملاً للأثر البيئي لمشروع تعديني واسع النطاق في منطقة غيتا.</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>شركة Geita Gold Mining Ltd</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>ОВОС для Горнодобывающего Проекта</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>Провели комплексную оценку воздействия на окружающую среду для крупномасштабного горнодобывающего проекта в регионе Гейта.</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>Geita Gold Mining Ltd</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>矿业项目环境影响评价</t>
-        </is>
-      </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>为盖塔地区一个大型矿业项目开展了全面的环境影响评价。</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>Geita Gold Mining Ltd</t>
-        </is>
-      </c>
+          <t>media/project_covers/WhatsApp_Image_2026-07-02_at_11.41.05_rkkqca</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>OHS Management System for Factory</t>
+          <t>ZEMD TANZANIA LIMITED</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ohs-factory</t>
+          <t>zemd-tanzania-limited</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Developed and implemented ISO 45001-compliant OHS management system for a manufacturing plant.</t>
+          <t>FeeVert Solution Limited provided ZEMD Tanzania Limited with an independent assessment of its environmental performance and compliance status, identifying environmental gaps and recommending corrective and preventive measures to strengthen environmental management and ensure continued compliance with relevant environmental requirements.
+This Compliance Environmental Audit demonstrates FeeVert's capacity and experience in providing professional environmental consultancy services to mining and industrial projects, including environmental audits, compliance monitoring, ESIA/EIA studies, environmental management planning, rehabilitation and closure planning, and environmental performance improvement.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ohs</t>
+          <t>environment</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Tanzania Manufacturers Ltd</t>
+          <t>ZEM Development Company Limited</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -7499,135 +7892,63 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>High incident rates and OSHA non-compliance</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Implemented OHSMS with training and monitoring</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Incidents reduced by 75%, OSHA compliance achieved</t>
-        </is>
-      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="b">
         <v>1</v>
       </c>
       <c r="K4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L4" t="b">
         <v>1</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>media/project_covers/TSF_PIC_3_php1pg</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Mfumo wa Usimamizi wa OHS kwa Kiwanda</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Tuliunda na kutekeleza mfumo wa usimamizi wa OHS unaozingatia ISO 45001 kwa kiwanda cha uzalishaji.</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Tanzania Manufacturers Ltd</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Système de Gestion SST pour une Usine</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>Développement et mise en œuvre d'un système de gestion SST conforme à la norme ISO 45001 pour une usine de fabrication.</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>Tanzania Manufacturers Ltd</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>نظام إدارة الصحة والسلامة المهنية لمصنع</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>طورنا ونفذنا نظام إدارة للصحة والسلامة المهنية متوافقًا مع ISO 45001 لمصنع تصنيع.</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>شركة Tanzania Manufacturers Ltd</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>Система Менеджмента ОТ для Завода</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>Разработали и внедрили систему менеджмента охраны труда, соответствующую ISO 45001, для производственного предприятия.</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>Tanzania Manufacturers Ltd</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>工厂职业健康安全管理体系</t>
-        </is>
-      </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>为一家制造工厂开发并实施了符合ISO 45001标准的职业健康安全管理体系。</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>Tanzania Manufacturers Ltd</t>
-        </is>
-      </c>
+          <t>media/project_covers/WhatsApp_Image_2026-06-25_at_08.43.00_5_xpcgia</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Honey Processing Facility Setup</t>
+          <t>OHS TRAINING AND COMPLIANCE AT XINCHENG DEVELOPMENT INVESTMENT COMPANY</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>honey-processing-facility</t>
+          <t>ohs-training-and-compliance-at-xincheng-development-investment-company</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Established a complete honey processing and packaging facility for a medium-scale beekeeper.</t>
+          <t>XINCHENG DEVELOPMENT INVESTMENT COMPANY IS A MINING COMPANY AND FEE-VERT SOLUTION LIMITED HAS MANAGED TO PROVIDE ENVIRONMENTAL AND SAFETY ENVIRONMENT FOR THE WORKERS BY PROVIDING EDUCATION, SAFETY ASSURANCE, COMPLIANCE ASSESSMENT OF THE COMPANY AND HEALTH GUIDANCE.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>beekeeping</t>
+          <t>ohs</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Morogoro Honey Processors</t>
+          <t>XINCHENG DEVELOPMENT INVESTMENT COMPANY</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -7635,135 +7956,63 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Lack of processing capacity and market access</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Built processing facility with TBS-compliant equipment</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Processing capacity increased 10x, export market access achieved</t>
-        </is>
-      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="b">
+        <v>1</v>
+      </c>
+      <c r="K5" t="n">
         <v>0</v>
       </c>
-      <c r="K5" t="n">
-        <v>4</v>
-      </c>
       <c r="L5" t="b">
         <v>1</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>media/project_covers/honey_bucket_pyyyj7</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Uanzishwaji wa Kituo cha Uchakataji wa Asali</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Tulianzisha kituo kamili cha uchakataji na ufungashaji wa asali kwa mfugaji nyuki wa kiwango cha kati.</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Morogoro Honey Processors</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>Installation d'une Unité de Transformation du Miel</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>Mise en place d'une unité complète de transformation et d'emballage du miel pour un apiculteur de taille moyenne.</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>Morogoro Honey Processors</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>إنشاء منشأة لمعالجة العسل</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>أنشأنا منشأة كاملة لمعالجة وتعبئة العسل لمربي نحل متوسط الحجم.</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>Morogoro Honey Processors</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>Создание Предприятия по Переработке Мёда</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>Создали полноценное предприятие по переработке и упаковке мёда для пчеловода среднего масштаба.</t>
-        </is>
-      </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>Morogoro Honey Processors</t>
-        </is>
-      </c>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>蜂蜜加工厂建设</t>
-        </is>
-      </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>为一位中等规模的养蜂人建立了完整的蜂蜜加工与包装设施。</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>Morogoro Honey Processors</t>
-        </is>
-      </c>
+          <t>media/project_covers/WhatsApp_Image_2026-09-25_at_08.59.20_vhmob4</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Environmental Audit for Hotel Chain</t>
+          <t>SUPPLY OF AGRICULTURAL IRRIGATION MONEY MAKER PUMPS</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>environmental-audit-hotel</t>
+          <t>supply-of-agricultural-irrigation-money-maker-pumps</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Annual environmental compliance audit for 5 hotels across Tanzania.</t>
+          <t>WORLD VISION IS AN INTERNATIONAL CHRISTIAN HUMANITARIAN ORGANIZATION DEDICATED TO WORKING WITH CHILDREN, FAMILIES AND COMMUNITIES TO OVERCOME POVERTY AND INJUSTICE. FEE-VERT SOLUTION LIMITED HAD A TENDER FOR THE SUPPLY OF AGRICULTURAL IRRIGATION PUMPS - MONEYMAKER PUMPS TO BARIADI AND KAHAMA.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>environment</t>
+          <t>agriculture</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Tanzania Hotels Group</t>
+          <t>WORLD VISION</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -7771,125 +8020,53 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Multiple sites with different environmental impacts</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Comprehensive audit with site-specific recommendations</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Full compliance achieved across all 5 sites</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="b">
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L6" t="b">
         <v>1</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>media/project_covers/environment-services01_qvblhq</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Ukaguzi wa Kimazingira kwa Mnyororo wa Hoteli</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Ukaguzi wa kila mwaka wa uzingatiaji wa kimazingira kwa hoteli 5 kote Tanzania.</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Tanzania Hotels Group</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>Audit Environnemental pour une Chaîne d'Hôtels</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>Audit annuel de conformité environnementale pour 5 hôtels à travers la Tanzanie.</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>Tanzania Hotels Group</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>تدقيق بيئي لسلسلة فنادق</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>تدقيق سنوي للامتثال البيئي لـ 5 فنادق في جميع أنحاء تنزانيا.</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>Tanzania Hotels Group</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>Экологический Аудит для Сети Отелей</t>
-        </is>
-      </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>Ежегодный аудит экологического соответствия для 5 отелей по всей Танзании.</t>
-        </is>
-      </c>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t>Tanzania Hotels Group</t>
-        </is>
-      </c>
-      <c r="Z6" t="inlineStr">
-        <is>
-          <t>酒店连锁环境审计</t>
-        </is>
-      </c>
-      <c r="AA6" t="inlineStr">
-        <is>
-          <t>为坦桑尼亚各地的5家酒店进行年度环境合规审计。</t>
-        </is>
-      </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>Tanzania Hotels Group</t>
-        </is>
-      </c>
+          <t>media/project_covers/WhatsApp_Image_2026-09-25_at_12.21.24_2_b7i1k5</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ESIA and Environmental Auditing for Xincheng Development Mining Company</t>
+          <t>YKKY MINING(T) CO. LIMITED</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>esia-environmental-auditing-xincheng-development-mining</t>
+          <t>ykky-miningt-co-limited</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>FeeVert Solution Limited had the pleasure of working with Xincheng Development Mining Co. Ltd. on the Environmental and Social Impact Assessment (ESIA), Environmental Compliance Audit, and Tailings Storage Facility (TSF) Audit for its mining project.</t>
+          <t>Fee-vert Solution Limited provided comprehensive consultancy services to YKKY Mining Co. Limited, supporting the development of its mining project through an integrated Environmental and Social Impact Assessment (ESIA), Feasibility Study, Resettlement Action Plan (RAP), Tailings Storage Facility (TSF) design, and Hydrogeological and Hydrological studies. Our multidisciplinary services were aimed at supporting technically sound, environmentally responsible, and socially sustainable project development.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -7899,7 +8076,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Xincheng Development Mining Company</t>
+          <t>YKKY COMPANY LIMITED</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -7907,242 +8084,442 @@
           <t>published</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>The project required coordinated ESIA, compliance audit, and TSF audit work under national environmental regulations and mining industry standards.</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Through our commitment to technical excellence, professionalism, and regulatory compliance, we conducted the ESIA, environmental compliance audit, and TSF audit in line with the required quality standards.</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>We successfully completed and delivered all assignments to the client's satisfaction, meeting the required quality standards and project timelines.</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="b">
         <v>1</v>
       </c>
       <c r="K7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L7" t="b">
         <v>1</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>media/project_covers/TSF_PIC_wwbv1s</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>ESIA na Ukaguzi wa Kimazingira kwa Kampuni ya Xincheng Development Mining</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>FeeVert Solution Limited ilipata fursa ya kufanya kazi na Xincheng Development Mining Co. Ltd. katika Tathmini ya Athari za Kimazingira na Kijamii (ESIA), Ukaguzi wa Uzingatiaji wa Kimazingira, na Ukaguzi wa Kituo cha Kuhifadhi Mabaki ya Madini (TSF) kwa mradi wake wa uchimbaji madini.</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>Xincheng Development Mining Company</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>EIES et Audit Environnemental pour Xincheng Development Mining Company</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>FeeVert Solution Limited a eu le plaisir de travailler avec Xincheng Development Mining Co. Ltd. sur l'Étude d'Impact Environnemental et Social (EIES), l'Audit de Conformité Environnementale, et l'Audit de l'Installation de Stockage des Résidus (TSF) pour son projet minier.</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>Xincheng Development Mining Company</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>تقييم الأثر البيئي والاجتماعي والتدقيق البيئي لشركة Xincheng Development Mining</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>كان من دواعي سرور شركة FeeVert Solution Limited العمل مع شركة Xincheng Development Mining Co. Ltd. في تقييم الأثر البيئي والاجتماعي، والتدقيق في الامتثال البيئي، وتدقيق منشأة تخزين المخلفات لمشروعها التعديني.</t>
-        </is>
-      </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>شركة Xincheng Development Mining</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>ЭСОВ и Экологический Аудит для Xincheng Development Mining Company</t>
-        </is>
-      </c>
-      <c r="X7" t="inlineStr">
-        <is>
-          <t>FeeVert Solution Limited имела удовольствие работать с Xincheng Development Mining Co. Ltd. над оценкой экологического и социального воздействия (ЭСОВ), аудитом экологического соответствия и аудитом хвостохранилища для её горнодобывающего проекта.</t>
-        </is>
-      </c>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>Xincheng Development Mining Company</t>
-        </is>
-      </c>
-      <c r="Z7" t="inlineStr">
-        <is>
-          <t>Xincheng Development Mining Company 环境社会影响评价与环境审计</t>
-        </is>
-      </c>
-      <c r="AA7" t="inlineStr">
-        <is>
-          <t>FeeVert Solution Limited 很荣幸与 Xincheng Development Mining Co. Ltd. 合作，为其矿业项目开展环境与社会影响评价（ESIA）、环境合规审计以及尾矿库（TSF）审计。</t>
-        </is>
-      </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>Xincheng Development Mining Company</t>
-        </is>
-      </c>
+          <t>media/project_covers/58660996-2e4d-4158-bf90-c015544fdfbe_qbjvzw</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>JIN CHUAN MINING CO. LIMITED</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>jin-chuan-mining-co-limited</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Fee-vert Solution Limited conducted a comprehensive Environmental and Social Impact Assessment (ESIA) for the RZ Union and Jin Chuan Mining Project, supporting the development of a large-scale mining operation. The assignment involved assessing potential environmental and social impacts associated with the proposed mining activities, developing appropriate mitigation and management measures, and ensuring compliance with applicable environmental and regulatory requirements. The assessment also supported responsible resource development, environmental protection, stakeholder considerations, and the promotion of sustainable mining practices throughout the project lifecycle.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>environment</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>RZ UNION MINING AND JIN CHUAN MINING COMPANY</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Complex regulatory requirements and community concerns</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Full ESIA with extensive stakeholder engagement</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>NEMC approval obtained, community agreement signed</t>
+        </is>
+      </c>
+      <c r="J8" t="b">
+        <v>1</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2</v>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>media/project_covers/GRAPHITE_MINING_PROJECT_lkomdi</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>EIA kwa Mradi wa Uchimbaji Madini</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Tulifanya Tathmini kamili ya Athari za Kimazingira kwa mradi mkubwa wa uchimbaji madini mkoani Geita.</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Geita Gold Mining Ltd</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>EIE pour un Projet Minier</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Réalisation d'une Étude d'Impact Environnemental complète pour un projet minier à grande échelle dans la région de Geita.</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Geita Gold Mining Ltd</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>تقييم الأثر البيئي لمشروع تعديني</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>أجرينا تقييمًا شاملاً للأثر البيئي لمشروع تعديني واسع النطاق في منطقة غيتا.</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>شركة Geita Gold Mining Ltd</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>ОВОС для Горнодобывающего Проекта</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>Провели комплексную оценку воздействия на окружающую среду для крупномасштабного горнодобывающего проекта в регионе Гейта.</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>Geita Gold Mining Ltd</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>矿业项目环境影响评价</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>为盖塔地区一个大型矿业项目开展了全面的环境影响评价。</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>Geita Gold Mining Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ESIA and Environmental Auditing for Xincheng Development Mining Company</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>esia-environmental-auditing-xincheng-development-mining</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>FeeVert Solution Limited had the pleasure of working with Xincheng Development Mining Co. Ltd. on the Environmental and Social Impact Assessment (ESIA), Environmental Compliance Audit, and Tailings Storage Facility (TSF) Audit for its mining project.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>environment</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>XINCHENG DEVELOPMENT MINING COMPANY</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>The project required coordinated ESIA, compliance audit, and TSF audit work under national environmental regulations and mining industry standards.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Through our commitment to technical excellence, professionalism, and regulatory compliance, we conducted the ESIA, environmental compliance audit, and TSF audit in line with the required quality standards.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>We successfully completed and delivered all assignments to the client's satisfaction, meeting the required quality standards and project timelines.</t>
+        </is>
+      </c>
+      <c r="J9" t="b">
+        <v>1</v>
+      </c>
+      <c r="K9" t="n">
+        <v>6</v>
+      </c>
+      <c r="L9" t="b">
+        <v>1</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>media/project_covers/TSF_PIC_wwbv1s</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>ESIA na Ukaguzi wa Kimazingira kwa Kampuni ya Xincheng Development Mining</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>FeeVert Solution Limited ilipata fursa ya kufanya kazi na Xincheng Development Mining Co. Ltd. katika Tathmini ya Athari za Kimazingira na Kijamii (ESIA), Ukaguzi wa Uzingatiaji wa Kimazingira, na Ukaguzi wa Kituo cha Kuhifadhi Mabaki ya Madini (TSF) kwa mradi wake wa uchimbaji madini.</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Xincheng Development Mining Company</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>EIES et Audit Environnemental pour Xincheng Development Mining Company</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>FeeVert Solution Limited a eu le plaisir de travailler avec Xincheng Development Mining Co. Ltd. sur l'Étude d'Impact Environnemental et Social (EIES), l'Audit de Conformité Environnementale, et l'Audit de l'Installation de Stockage des Résidus (TSF) pour son projet minier.</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Xincheng Development Mining Company</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>تقييم الأثر البيئي والاجتماعي والتدقيق البيئي لشركة Xincheng Development Mining</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>كان من دواعي سرور شركة FeeVert Solution Limited العمل مع شركة Xincheng Development Mining Co. Ltd. في تقييم الأثر البيئي والاجتماعي، والتدقيق في الامتثال البيئي، وتدقيق منشأة تخزين المخلفات لمشروعها التعديني.</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>شركة Xincheng Development Mining</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>ЭСОВ и Экологический Аудит для Xincheng Development Mining Company</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>FeeVert Solution Limited имела удовольствие работать с Xincheng Development Mining Co. Ltd. над оценкой экологического и социального воздействия (ЭСОВ), аудитом экологического соответствия и аудитом хвостохранилища для её горнодобывающего проекта.</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>Xincheng Development Mining Company</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>Xincheng Development Mining Company 环境社会影响评价与环境审计</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>FeeVert Solution Limited 很荣幸与 Xincheng Development Mining Co. Ltd. 合作，为其矿业项目开展环境与社会影响评价（ESIA）、环境合规审计以及尾矿库（TSF）审计。</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>Xincheng Development Mining Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Commercial Langstroth Beehive Supply for World Vision</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>commercial-langstroth-beehive-supply-world-vision</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Supply of commercial Langstroth beehives for beekeeping and environmental conservation, supporting World Vision's community livelihood and conservation programs.</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Fee-vert Solution Limited supplied commercial Langstroth beehives for beekeeping and environmental conservation, supporting World Vision's community livelihood and conservation programs.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
         <is>
           <t>beekeeping</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>WORLD VISION</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>The programme needed durable, commercial-grade beehives suited to local conditions to support beekeeping-based livelihoods and environmental conservation.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Fee-vert Solution Limited supplied commercial Langstroth beehives, drawing on bees' role in honey and beeswax production, pollen production, and improved crop pollination for better crop management and crop rotation.</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>The beehives were delivered and installed to support beekeeping-based community livelihoods alongside environmental conservation goals.</t>
+        </is>
+      </c>
+      <c r="J10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K10" t="n">
+        <v>7</v>
+      </c>
+      <c r="L10" t="b">
+        <v>1</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>media/project_covers/COMMERCIAL_LANGSTROTH_BEEHIVE_khrbtc</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Ugavi wa Mizinga ya Kibiashara ya Langstroth kwa World Vision</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Ugavi wa mizinga ya kibiashara ya Langstroth kwa ajili ya ufugaji nyuki na uhifadhi wa mazingira, ikisaidia mipango ya World Vision ya kipato cha jamii na uhifadhi.</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
         <is>
           <t>World Vision</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>published</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>The programme needed durable, commercial-grade beehives suited to local conditions to support beekeeping-based livelihoods and environmental conservation.</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>FeeVert supplied commercial Langstroth beehives, drawing on bees' role in honey and beeswax production, pollen production, and improved crop pollination for better crop management and crop rotation.</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>The beehives were delivered and installed to support beekeeping-based community livelihoods alongside environmental conservation goals.</t>
-        </is>
-      </c>
-      <c r="J8" t="b">
-        <v>1</v>
-      </c>
-      <c r="K8" t="n">
-        <v>7</v>
-      </c>
-      <c r="L8" t="b">
-        <v>1</v>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>media/project_covers/COMMERCIAL_LANGSTROTH_BEEHIVE_khrbtc</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>Ugavi wa Mizinga ya Kibiashara ya Langstroth kwa World Vision</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>Ugavi wa mizinga ya kibiashara ya Langstroth kwa ajili ya ufugaji nyuki na uhifadhi wa mazingira, ikisaidia mipango ya World Vision ya kipato cha jamii na uhifadhi.</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Fourniture de Ruches Langstroth Commerciales pour World Vision</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Fourniture de ruches Langstroth commerciales pour l'apiculture et la conservation environnementale, soutenant les programmes de moyens de subsistance communautaires et de conservation de World Vision.</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
         <is>
           <t>World Vision</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>Fourniture de Ruches Langstroth Commerciales pour World Vision</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>Fourniture de ruches Langstroth commerciales pour l'apiculture et la conservation environnementale, soutenant les programmes de moyens de subsistance communautaires et de conservation de World Vision.</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>توريد خلايا لانغستروث التجارية لمنظمة World Vision</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>توريد خلايا لانغستروث التجارية لتربية النحل والحفاظ على البيئة، دعمًا لبرامج منظمة World Vision الخاصة بسبل العيش المجتمعية والحفاظ على البيئة.</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
         <is>
           <t>World Vision</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>توريد خلايا لانغستروث التجارية لمنظمة World Vision</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>توريد خلايا لانغستروث التجارية لتربية النحل والحفاظ على البيئة، دعمًا لبرامج منظمة World Vision الخاصة بسبل العيش المجتمعية والحفاظ على البيئة.</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr">
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Поставка Коммерческих Ульев Лангстрота для World Vision</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>Поставка коммерческих ульев Лангстрота для пчеловодства и охраны окружающей среды в поддержку программ World Vision по обеспечению средств к существованию сообществ и охране природы.</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
         <is>
           <t>World Vision</t>
         </is>
       </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>Поставка Коммерческих Ульев Лангстрота для World Vision</t>
-        </is>
-      </c>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t>Поставка коммерческих ульев Лангстрота для пчеловодства и охраны окружающей среды в поддержку программ World Vision по обеспечению средств к существованию сообществ и охране природы.</t>
-        </is>
-      </c>
-      <c r="Y8" t="inlineStr">
-        <is>
-          <t>World Vision</t>
-        </is>
-      </c>
-      <c r="Z8" t="inlineStr">
+      <c r="Z10" t="inlineStr">
         <is>
           <t>为 World Vision 提供商业朗氏蜂箱供应</t>
         </is>
       </c>
-      <c r="AA8" t="inlineStr">
+      <c r="AA10" t="inlineStr">
         <is>
           <t>供应商业朗氏蜂箱用于养蜂及环境保护，支持 World Vision 的社区生计与保护项目。</t>
         </is>
       </c>
-      <c r="AB8" t="inlineStr">
+      <c r="AB10" t="inlineStr">
         <is>
           <t>World Vision</t>
         </is>
@@ -8292,7 +8669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S4"/>
+  <dimension ref="A1:S9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8395,12 +8772,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ENDREWCUS JOHN MASERO</t>
+          <t>GODLOVE U.J. MWAMSOJO</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Managing Director &amp; Registered Environmental Expert</t>
+          <t>Senior Environmental Consultant</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -8410,76 +8787,35 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Endrewcus John Masero is the Founder and Managing Director of FEE-VERT SOLUTION LIMITED, a leading environmental consultancy firm in Tanzania. He is a Registered Environmental Expert with NEMC (NEMC/EA/0188) holding a Bachelor's degree in Environmental Sciences and Management from Sokoine University of Agriculture. With over 15 years of cross-sectoral experience spanning mining, construction, pharmaceuticals, and environmental management, Endrewcus brings strategic leadership and technical excellence to every project. He is certified in ISO 14001 Environmental Management Systems and OHSAS 18001 Occupational Health &amp; Safety.</t>
+          <t>Mr. Mwamsojo is a Senior Environmental Consultant with extensive professional experience in environmental management. He is a registered and accredited expert in Environmental Impact Assessment (EIA) and Environmental Auditing (EA) in accordance with the Environmental Management Act No. 191 of 2004. He has participated in numerous environmental projects, providing technical leadership, mentoring environmental trainees, and overseeing on-site project implementation.
+Mr. Mwamsojo possesses strong hands-on experience with advanced analytical, data processing, and decision-support tools applied across multiple disciplines. His technical expertise includes the use of Microsoft Office applications, GIS and remote sensing technologies, as well as modeling tools for hydraulics, surface/groundwater systems, industrial and municipal wastewater, air quality, river basin management, and flood risk analysis.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>endrewcus.masero@feevert.co.tz</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>2557685603080</v>
-      </c>
+          <t>mwamsonjo@feevert.co.tz</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I2" t="b">
         <v>1</v>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Mkurugenzi Mtendaji na Mtaalamu wa Mazingira Aliyesajiliwa</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Endrewcus John Masero ni Mwanzilishi na Mkurugenzi Mtendaji wa FEE-VERT SOLUTION LIMITED, kampuni inayoongoza kwa ushauri wa kimazingira nchini Tanzania. Ni Mtaalamu wa Mazingira Aliyesajiliwa na NEMC (NEMC/EA/0188) mwenye shahada ya kwanza katika Sayansi na Usimamizi wa Mazingira kutoka Chuo Kikuu cha Kilimo cha Sokoine. Akiwa na uzoefu wa zaidi ya miaka 15 katika sekta mbalimbali ikiwemo uchimbaji madini, ujenzi, dawa, na usimamizi wa mazingira, Endrewcus analeta uongozi wa kimkakati na ubora wa kitaalamu katika kila mradi. Ana vyeti vya Mifumo ya Usimamizi wa Mazingira ya ISO 14001 na Afya na Usalama Mahali pa Kazi ya OHSAS 18001.</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Directeur Général &amp; Expert Environnemental Agréé</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Endrewcus John Masero est le Fondateur et Directeur Général de FEE-VERT SOLUTION LIMITED, un cabinet de conseil environnemental de premier plan en Tanzanie. Il est Expert Environnemental Agréé auprès du NEMC (NEMC/EA/0188), titulaire d'une licence en Sciences et Gestion de l'Environnement de l'Université d'Agriculture de Sokoine. Avec plus de 15 ans d'expérience intersectorielle couvrant les mines, la construction, la pharmacie, et la gestion environnementale, Endrewcus apporte un leadership stratégique et une excellence technique à chaque projet. Il est certifié en Systèmes de Management Environnemental ISO 14001 et en Santé et Sécurité au Travail OHSAS 18001.</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>المدير التنفيذي وخبير بيئي مسجل</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>إندريوكس جون ماسيرو هو المؤسس والمدير التنفيذي لشركة FEE-VERT SOLUTION LIMITED، إحدى الشركات الاستشارية البيئية الرائدة في تنزانيا. وهو خبير بيئي مسجل لدى المجلس الوطني لإدارة البيئة (NEMC/EA/0188)، حاصل على درجة البكالوريوس في العلوم البيئية والإدارة من جامعة سوكوين للزراعة. وبخبرة تزيد عن 15 عامًا في قطاعات متعددة تشمل التعدين والبناء والصيدلة والإدارة البيئية، يقدم إندريوكس قيادة استراتيجية وتميزًا تقنيًا في كل مشروع. وهو حاصل على شهادات في أنظمة الإدارة البيئية ISO 14001 والصحة والسلامة المهنية OHSAS 18001.</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Управляющий директор и зарегистрированный эксперт-эколог</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>Эндрюкус Джон Масеро — основатель и управляющий директор компании FEE-VERT SOLUTION LIMITED, ведущей экологической консалтинговой компании в Танзании. Он является зарегистрированным экспертом-экологом при NEMC (NEMC/EA/0188), имеет степень бакалавра в области экологических наук и управления окружающей средой Сельскохозяйственного университета Сокойне. Обладая более чем 15-летним межотраслевым опытом в горнодобывающей, строительной, фармацевтической и природоохранной сферах, Эндрюкус привносит стратегическое руководство и техническое совершенство в каждый проект. Он сертифицирован по системам экологического менеджмента ISO 14001 и охране труда и технике безопасности OHSAS 18001.</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>董事总经理兼注册环境专家</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>Endrewcus John Masero 是 FEE-VERT SOLUTION LIMITED 的创始人兼董事总经理，该公司是坦桑尼亚领先的环境咨询公司。他是国家环境管理委员会（NEMC）注册环境专家（编号：NEMC/EA/0188），拥有索科伊内农业大学环境科学与管理学士学位。他拥有超过15年跨行业经验，涵盖采矿、建筑、制药和环境管理领域，为每个项目带来战略领导力和卓越的技术能力。他持有ISO 14001环境管理体系和OHSAS 18001职业健康安全认证。</t>
-        </is>
-      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8489,7 +8825,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Director General</t>
+          <t>Senior Agro-Ecologist Researcher</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8507,7 +8843,11 @@
           <t>essau.losujaki@feevert.co.tz</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G3" t="b">
         <v>1</v>
       </c>
@@ -8571,89 +8911,341 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NICOLE ABBAS MOHAMED</t>
+          <t>YESAYA WILLIAM KAONEKA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ENVIRONMENTAL ENGINEER</t>
+          <t>Senior Environmental Consultant</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Consulting</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Nicole Abbas Mohamed is an Environmental Engineer with a strong academic background, including a dissertation on environmental sustainability, contributing to the company's environmental management and monitoring initiatives.</t>
+          <t>Mr. Kaoneka holds a Bachelor of Science in Environmental Science from Ardhi University and is a registered Environmental Expert with over 11 years of professional experience in Environmental Health and Safety. His core competencies include Environmental Impact Assessment and Auditing, enforcement of OSHA and EMA regulations, risk assessment, waste management, and supervision of safe working environments. He is a self-motivated professional with strong analytical and problem-solving skills, recognized for developing innovative and practical solutions to environmental health and safety challenges in the workplace.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>nicole.mohamed@feevert.co.tz</t>
+          <t>kaoneka@feevert.co.tz</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DENIS NYAMBELE BONIFACE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Civil Engineer</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Consulting</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Mr. Denis is a registered Professional Engineer (PE) with experience in civil engineering and surveying multiple infrastructure projects. He is responsible for supervising site works, desk and field assignments, reconnaissance surveys, laboratory testing programs, interpretation of test results, and technical reporting. He is an enthusiastic and resolute professional with strong practical and technical capabilities.
+His former professional experience includes roles as a Technician and Surveyor at China Civil Engineering Construction Corporation (CCECC), Material Engineer and Supervisor at Mohammedi Builders Limited, and Civil Engineer and Surveyor at ICE Project Services. He brings a strong multidisciplinary background that supports effective project delivery and quality assurance.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>denis.nyambele@feevert.co.tz</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I5" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>FRANSISCO JOHN CYPRIAN</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Geologist</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Mr. Fransisco is a graduate in Geology from the University of Dar es Salaam with over three years of professional experience in exploration geology. He has developed strong, hands-on expertise in mineral exploration and geological mapping across Tanzania, with a particular focus on copper exploration from early-stage target generation to resource definition. His technical competencies include geological and structural mapping, geochemical and geophysical surveys (magnetometer and IP/resistivity), core drilling supervision, and geological modeling. He is proficient in ArcGIS, Supak, and MapInfo for data analysis, interpretation, and visualization. Mr. Fransisco has in-depth knowledge of major geological terrains in Tanzania, including the Dodoma Terrane, Mpanda, Chunya, Geita, Mwanza, Shinyanga, and Lindi, and a strong understanding of their copper mineralization potential. His ability to integrate geological, geochemical, and geophysical datasets enables effective identification and delineation of mineralized zones. His geological expertise is also critical in supporting geotechnical, hydrogeological, and feasibility studies for mining investments.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>fransisco@feevert.co.tz</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>5</v>
+      </c>
+      <c r="I6" t="b">
+        <v>1</v>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PRISILA PIUS NEEMA</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Prisila Pius is an experienced Accountant with a Bachelor of Science in Taxation. She is responsible for managing the company’s financial affairs, including accounting, financial reporting, budgeting, cash-flow management, tax compliance and financial records. Her strong taxation background enables her to effectively manage financial and statutory requirements while promoting accuracy, transparency, accountability, and sound financial management within the organization.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>prisila.neema@feevert.co.tz</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>+255 719 030 567</t>
+        </is>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
         <v>6</v>
       </c>
-      <c r="I4" t="b">
-        <v>1</v>
-      </c>
-      <c r="J4" t="inlineStr">
+      <c r="I7" t="b">
+        <v>1</v>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>NICOLE ABBAS MOHAMED</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Environmental Manager</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Nicole Abbas Mohamed is an Environmental Engineering professional with practical experience in Environmental and Social Impact Assessments (ESIA), environmental compliance, occupational safety and health, construction-site inspection, water and sanitation systems, and sustainable development. She holds a Bachelor of Science in Environmental Engineering from Ardhi University (awarded December 2025). 
+Her professional experience includes supporting environmental activities for mining and development projects, conducting site inspections, identifying environmental and workplace risks, preparing technical documentation, and contributing to sustainable solutions.
+Nicole is a proactive, analytical, and collaborative professional who prioritizes environmental responsibility, workplace safety, continuous learning, and meaningful stakeholder engagement. Proficient in key analytical and data tools such as SPSS and MS Office, she brings hands-on experience in water systems design, construction supervision, and rural water supply to every project. Nicole is dedicated to advancing sustainable environmental management and community development initiatives across diverse sectors.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>nicole.abbas@feevert.co.tz</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>+255624012055</t>
+        </is>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>7</v>
+      </c>
+      <c r="I8" t="b">
+        <v>1</v>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>Mhandisi wa Mazingira</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>Nicole Abbas Mohamed ni Mhandisi wa Mazingira mwenye msingi thabiti wa kitaaluma, ikiwemo tasnifu kuhusu uendelevu wa mazingira, akichangia katika mipango ya usimamizi na ufuatiliaji wa mazingira wa kampuni.</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>Ingénieure Environnementale</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>Nicole Abbas Mohamed est Ingénieure Environnementale avec un solide parcours académique, incluant un mémoire sur la durabilité environnementale, contribuant aux initiatives de gestion et de suivi environnemental de l'entreprise.</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>مهندسة بيئية</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>نيكول عباس محمد مهندسة بيئية ذات خلفية أكاديمية قوية، بما في ذلك أطروحة حول الاستدامة البيئية، تساهم في مبادرات إدارة ومراقبة البيئة الخاصة بالشركة.</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>Инженер-эколог</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>Николь Аббас Мохамед — инженер-эколог с солидной академической подготовкой, включая диссертацию по экологической устойчивости, вносящий вклад в инициативы компании по экологическому менеджменту и мониторингу.</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>环境工程师</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>Nicole Abbas Mohamed 是一位拥有扎实学术背景的环境工程师，曾撰写关于环境可持续性的论文，为公司的环境管理与监测项目做出贡献。</t>
         </is>
       </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SAIDINA RIDHIWANI RASHIDI</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Safety officer</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Saidina Ridhiwani Rashidi is an Environmental and Occupational Health and Safety professional with an academic background in Geography and Environmental Studies from the University of Dar es Salaam.
+She brings a strong understanding of environmental management, workplace safety, risk prevention, and organizational wellbeing. In her role, she supports the implementation of Occupational Health and Safety standards within the office environment with a focus on maintaining safe working conditions, strengthening compliance with internal safety procedures, identifying workplace risks and promoting a proactive safety culture across the organization.
+Her professional approach integrates environmental awareness, occupational safety and responsible workplace practices to support operational efficiency and employee wellbeing. She is committed to strengthening systems and practices that contribute to a safe, compliant and sustainable working environment.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>saidina@feevert.co.tz</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0715745866</t>
+        </is>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>8</v>
+      </c>
+      <c r="I9" t="b">
+        <v>1</v>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8849,7 +9441,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>FeeVert is a professional consultancy firm providing expert services in  Environmental Consultancy, Sustainable Agriculture &amp; Commercial Beekeeping, and Occupational Health &amp; Safety (OHS).</t>
+          <t>FEE-VERT SOLUTION LIMITED is a professional Tanzanian consultancy and services firm dedicated to delivering innovative, sustainable, and practical solutions across Environmental Consultancy, Sustainable Agriculture &amp; Commercial Beekeeping, and Occupational Health &amp; Safety (OHS).</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -9124,7 +9716,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>media/hero/environment-services01_ntslq8</t>
+          <t>media/hero/GRAPHITE_MINING_PROJECT_hvq7dk</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">

</xml_diff>